<commit_message>
Preparar AsistenteBodegaIA para despliegue en Vercel
</commit_message>
<xml_diff>
--- a/datos/medidas_discos.xlsx
+++ b/datos/medidas_discos.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS TUF F15\Desktop\AsistenteBodegaIA\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{105A1700-1925-4889-A951-E14913112022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF55045-C129-4006-9AD3-294199BCB8FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{14E3A02E-E182-494D-BF65-FBDEDAC9F4E2}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId2"/>
+    <externalReference r:id="rId3"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja2!$A$1:$H$898</definedName>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3317" uniqueCount="1083">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3321" uniqueCount="1083">
   <si>
     <t>CODIGO</t>
   </si>
@@ -3602,9 +3603,11 @@
           </cell>
         </row>
         <row r="10">
+          <cell r="C10"/>
           <cell r="D10" t="str">
             <v>J52-3501075</v>
           </cell>
+          <cell r="E10"/>
           <cell r="F10" t="str">
             <v>Disco Freno Cerry Arrizo 3</v>
           </cell>
@@ -3628,6 +3631,7 @@
           </cell>
         </row>
         <row r="11">
+          <cell r="C11"/>
           <cell r="D11" t="str">
             <v>J603502075</v>
           </cell>
@@ -3689,9 +3693,11 @@
           </cell>
         </row>
         <row r="13">
+          <cell r="C13"/>
           <cell r="D13" t="str">
             <v>T15-3501075</v>
           </cell>
+          <cell r="E13"/>
           <cell r="F13" t="str">
             <v>Disco Freno Cherry Tiggo 4 7 8, Tiggo 8 Pro 1.5 1.6 16&gt;</v>
           </cell>
@@ -3721,6 +3727,7 @@
           <cell r="D14" t="str">
             <v>3501101-CA01</v>
           </cell>
+          <cell r="E14"/>
           <cell r="F14" t="str">
             <v>Disco Freno Dfsk Glory 580 / Mini van C37 1.5 18-24</v>
           </cell>
@@ -3782,6 +3789,7 @@
           <cell r="D16" t="str">
             <v>35G01</v>
           </cell>
+          <cell r="E16"/>
           <cell r="F16" t="str">
             <v>Disco Freno Shineray SWM G01 19-24</v>
           </cell>
@@ -3805,6 +3813,8 @@
           </cell>
         </row>
         <row r="17">
+          <cell r="C17"/>
+          <cell r="D17"/>
           <cell r="E17" t="str">
             <v>HF - 9466</v>
           </cell>
@@ -3831,6 +3841,8 @@
           </cell>
         </row>
         <row r="18">
+          <cell r="C18"/>
+          <cell r="D18"/>
           <cell r="E18" t="str">
             <v>HF - 9441</v>
           </cell>
@@ -3857,6 +3869,8 @@
           </cell>
         </row>
         <row r="19">
+          <cell r="C19"/>
+          <cell r="D19"/>
           <cell r="E19" t="str">
             <v>HF - 9440</v>
           </cell>
@@ -3883,6 +3897,8 @@
           </cell>
         </row>
         <row r="20">
+          <cell r="C20"/>
+          <cell r="D20"/>
           <cell r="E20" t="str">
             <v>HF - 9473</v>
           </cell>
@@ -3909,6 +3925,8 @@
           </cell>
         </row>
         <row r="21">
+          <cell r="C21"/>
+          <cell r="D21"/>
           <cell r="E21" t="str">
             <v>HF - 9469</v>
           </cell>
@@ -3935,9 +3953,11 @@
           </cell>
         </row>
         <row r="22">
+          <cell r="C22"/>
           <cell r="D22" t="str">
             <v>23B02A024</v>
           </cell>
+          <cell r="E22"/>
           <cell r="F22" t="str">
             <v>Disco Freno Soueast DX7 Prime 1.5 2.020</v>
           </cell>
@@ -3967,6 +3987,7 @@
           <cell r="D23" t="str">
             <v>S213501075</v>
           </cell>
+          <cell r="E23"/>
           <cell r="F23" t="str">
             <v>Disco Freno Cherry Practivan QQ6 Van Pass N300</v>
           </cell>
@@ -4988,6 +5009,7 @@
           <cell r="D55" t="str">
             <v>3501011-S08</v>
           </cell>
+          <cell r="E55"/>
           <cell r="F55" t="str">
             <v>Disco Freno Great Wall Hover M4 1.5 14-21</v>
           </cell>
@@ -5043,6 +5065,8 @@
           </cell>
         </row>
         <row r="57">
+          <cell r="C57"/>
+          <cell r="D57"/>
           <cell r="E57" t="str">
             <v>HF - 9468</v>
           </cell>
@@ -5069,6 +5093,8 @@
           </cell>
         </row>
         <row r="58">
+          <cell r="C58"/>
+          <cell r="D58"/>
           <cell r="E58" t="str">
             <v>HF - 9470</v>
           </cell>
@@ -5194,6 +5220,7 @@
           <cell r="C62" t="str">
             <v>BD6041</v>
           </cell>
+          <cell r="D62"/>
           <cell r="E62" t="str">
             <v>HF - 302C</v>
           </cell>
@@ -5252,6 +5279,7 @@
           </cell>
         </row>
         <row r="64">
+          <cell r="C64"/>
           <cell r="D64" t="str">
             <v>5531160B22</v>
           </cell>
@@ -5569,9 +5597,11 @@
           </cell>
         </row>
         <row r="74">
+          <cell r="C74"/>
           <cell r="D74">
             <v>23995887</v>
           </cell>
+          <cell r="E74"/>
           <cell r="F74" t="str">
             <v xml:space="preserve">Disco Freno Chevrolet Captiva Turbo 1.5 </v>
           </cell>
@@ -5595,9 +5625,11 @@
           </cell>
         </row>
         <row r="75">
+          <cell r="C75"/>
           <cell r="D75">
             <v>23960473</v>
           </cell>
+          <cell r="E75"/>
           <cell r="F75" t="str">
             <v xml:space="preserve">Disco Freno Chevrolet Captiva LTZ Turbo 1.5 5P 2023 </v>
           </cell>
@@ -5621,9 +5653,11 @@
           </cell>
         </row>
         <row r="76">
+          <cell r="C76"/>
           <cell r="D76">
             <v>23971417</v>
           </cell>
+          <cell r="E76"/>
           <cell r="F76" t="str">
             <v xml:space="preserve">Disco Freno Chevrolet Captiva Turbo 1.5 </v>
           </cell>
@@ -5938,6 +5972,7 @@
           <cell r="C86" t="str">
             <v>BD2561</v>
           </cell>
+          <cell r="D86"/>
           <cell r="E86" t="str">
             <v>HF - 9343</v>
           </cell>
@@ -6287,6 +6322,7 @@
           <cell r="C97" t="str">
             <v>BD0570</v>
           </cell>
+          <cell r="D97"/>
           <cell r="E97" t="str">
             <v>HF - 102F</v>
           </cell>
@@ -6348,6 +6384,8 @@
           <cell r="C99" t="str">
             <v>BD7510</v>
           </cell>
+          <cell r="D99"/>
+          <cell r="E99"/>
           <cell r="F99" t="str">
             <v>Disco Freno Hyundai Grna I10 1.2 14&gt;</v>
           </cell>
@@ -6674,6 +6712,11 @@
           <cell r="G109" t="str">
             <v>V/D</v>
           </cell>
+          <cell r="H109"/>
+          <cell r="I109"/>
+          <cell r="J109"/>
+          <cell r="K109"/>
+          <cell r="L109"/>
         </row>
         <row r="110">
           <cell r="C110" t="str">
@@ -6772,6 +6815,9 @@
           </cell>
         </row>
         <row r="113">
+          <cell r="C113"/>
+          <cell r="D113"/>
+          <cell r="E113"/>
           <cell r="F113" t="str">
             <v>Disco Freno Hyundai Tucson 2.0 21-23, Kia Sportage 2.0 21-23</v>
           </cell>
@@ -6923,6 +6969,8 @@
           </cell>
         </row>
         <row r="118">
+          <cell r="C118"/>
+          <cell r="D118"/>
           <cell r="E118" t="str">
             <v>HF - 9436</v>
           </cell>
@@ -6949,6 +6997,8 @@
           </cell>
         </row>
         <row r="119">
+          <cell r="C119"/>
+          <cell r="D119"/>
           <cell r="E119" t="str">
             <v>HF - 9437</v>
           </cell>
@@ -7205,6 +7255,7 @@
           <cell r="D127" t="str">
             <v>51712-G6000</v>
           </cell>
+          <cell r="E127"/>
           <cell r="F127" t="str">
             <v xml:space="preserve">Disco Freno Kia Picanto1.0 G3LA HB-5P, 1.2  G4LA HB-5P 20-24 </v>
           </cell>
@@ -7234,6 +7285,7 @@
           <cell r="D128" t="str">
             <v>51712-G6300</v>
           </cell>
+          <cell r="E128"/>
           <cell r="F128" t="str">
             <v xml:space="preserve">Disco Freno Kia Picanto1.0 G3LA HB-5P, 1.2 G4LA HB-5P 17-20  </v>
           </cell>
@@ -7551,6 +7603,7 @@
           <cell r="D138" t="str">
             <v>BDWK33251</v>
           </cell>
+          <cell r="E138"/>
           <cell r="F138" t="str">
             <v>Disco Freno Mazda CX-30 2.0 5P 4X2 TM</v>
           </cell>
@@ -7638,6 +7691,8 @@
           </cell>
         </row>
         <row r="141">
+          <cell r="C141"/>
+          <cell r="D141"/>
           <cell r="E141" t="str">
             <v>HF - 867A</v>
           </cell>
@@ -7827,6 +7882,8 @@
           <cell r="C147" t="str">
             <v>BD3565</v>
           </cell>
+          <cell r="D147"/>
+          <cell r="E147"/>
           <cell r="F147" t="str">
             <v>Disco Freno Mazda 3 2.0 13-19 / Mazda CX3 2.0 15-23</v>
           </cell>
@@ -8234,6 +8291,7 @@
           </cell>
         </row>
         <row r="160">
+          <cell r="C160"/>
           <cell r="D160" t="str">
             <v>4615A125/CA350135</v>
           </cell>
@@ -8554,6 +8612,8 @@
           <cell r="C170" t="str">
             <v>BD1158</v>
           </cell>
+          <cell r="D170"/>
+          <cell r="E170"/>
           <cell r="F170" t="str">
             <v>Disco Freno Nissan Frontier CS XE CD SE 2.8 02-08 (Diesel)  (EG)</v>
           </cell>
@@ -8807,6 +8867,7 @@
           <cell r="D178" t="str">
             <v>40206T01A</v>
           </cell>
+          <cell r="E178"/>
           <cell r="F178" t="str">
             <v>Disco Freno Nissan X-Trail T30 2.0 2.5 23&gt;, Qashqai 2.0 2.5 23&gt;</v>
           </cell>
@@ -9921,6 +9982,7 @@
           <cell r="C213" t="str">
             <v>BD4137</v>
           </cell>
+          <cell r="D213"/>
           <cell r="E213" t="str">
             <v>HF - 507A</v>
           </cell>
@@ -10139,6 +10201,7 @@
           </cell>
         </row>
         <row r="220">
+          <cell r="C220"/>
           <cell r="D220">
             <v>4351206090</v>
           </cell>
@@ -10206,6 +10269,7 @@
           <cell r="D222" t="str">
             <v>43512-OK170</v>
           </cell>
+          <cell r="E222"/>
           <cell r="F222" t="str">
             <v>Disco Freno Toyota Hilux 2.7 4X2 16-22</v>
           </cell>
@@ -10261,6 +10325,7 @@
           </cell>
         </row>
         <row r="224">
+          <cell r="C224"/>
           <cell r="D224" t="str">
             <v>43512OK220</v>
           </cell>
@@ -10322,9 +10387,11 @@
           </cell>
         </row>
         <row r="226">
+          <cell r="C226"/>
           <cell r="D226" t="str">
             <v>3504300P33A0</v>
           </cell>
+          <cell r="E226"/>
           <cell r="F226" t="str">
             <v>Disco Freno Jac T6 T8 2.0 4X2 4X4</v>
           </cell>
@@ -10380,6 +10447,7 @@
           </cell>
         </row>
         <row r="228">
+          <cell r="C228"/>
           <cell r="D228" t="str">
             <v>431520K280</v>
           </cell>
@@ -10409,6 +10477,8 @@
           </cell>
         </row>
         <row r="229">
+          <cell r="C229"/>
+          <cell r="D229"/>
           <cell r="E229" t="str">
             <v>HF - 9438</v>
           </cell>
@@ -10534,6 +10604,8 @@
           <cell r="C233" t="str">
             <v>BD3392</v>
           </cell>
+          <cell r="D233"/>
+          <cell r="E233"/>
           <cell r="F233" t="str">
             <v xml:space="preserve">Disco Freno Volks Golf - Passat 1.3 93&lt; </v>
           </cell>
@@ -35304,4 +35376,40 @@
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66FBBB6B-5BBB-4C4A-B6EE-79B7F6B1A14F}">
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>410</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="4">
+        <v>262</v>
+      </c>
+      <c r="E1" s="4">
+        <v>10</v>
+      </c>
+      <c r="F1" s="4">
+        <v>45</v>
+      </c>
+      <c r="G1" s="4">
+        <v>76</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>